<commit_message>
Update Inventory and Master Plan docs for Form Submissions automation
Inventory sheet: Form Submissions row now shows Partial Coverage (29/51)
with real Tests Automated/Not Automatable counts (was TBD placeholder);
TOTAL row recalculated to include it (248/143, 63.4% automated - also drops
the now-outdated "excl. Form Submissions" caveat).

Master Plan: added the same Maestro Automatability / Automated? / Flow File
columns (I/J/K) used in every other automated tab to the Form Submissions
tab, populated by matching Test Case ID against coverage_matrix.csv (all 51
rows matched exactly; the 4 section-header rows are correctly left blank).
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -6471,12 +6471,12 @@
 (Yes / Partial Coverage / No / N/A)</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="0" t="inlineStr">
         <is>
           <t>Tests Automated (Count)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="0" t="inlineStr">
         <is>
           <t>Not Automatable (Count)</t>
         </is>
@@ -6519,10 +6519,10 @@
           <t>N/A - manual, out of scope for Maestro</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="0" t="n">
         <v>35</v>
       </c>
     </row>
@@ -6559,10 +6559,10 @@
           <t>Partial Coverage (6/7)</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="K6" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6595,10 +6595,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="K7" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="L7" t="n">
+      <c r="L7" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6635,10 +6635,10 @@
           <t>Partial Coverage (7/14)</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="K8" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="L8" t="n">
+      <c r="L8" s="0" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6671,10 +6671,10 @@
           <t>Partial Coverage (21/22)</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="K9" s="0" t="n">
         <v>21</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L9" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6711,10 +6711,10 @@
           <t>Partial Coverage (48/66)</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="K10" s="0" t="n">
         <v>48</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L10" s="0" t="n">
         <v>22</v>
       </c>
     </row>
@@ -6747,10 +6747,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="K11" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="L11" t="n">
+      <c r="L11" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6783,10 +6783,10 @@
           <t>Partial Coverage (4/13)</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="K12" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="L12" t="n">
+      <c r="L12" s="0" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6819,10 +6819,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="K13" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="L13" t="n">
+      <c r="L13" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6855,10 +6855,10 @@
           <t>Partial Coverage (6/8)</t>
         </is>
       </c>
-      <c r="K14" t="n">
+      <c r="K14" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="L14" t="n">
+      <c r="L14" s="0" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6891,10 +6891,10 @@
           <t>Partial Coverage (11/13)</t>
         </is>
       </c>
-      <c r="K15" t="n">
+      <c r="K15" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="L15" t="n">
+      <c r="L15" s="0" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6927,10 +6927,10 @@
           <t>Partial Coverage (4/5)</t>
         </is>
       </c>
-      <c r="K16" t="n">
+      <c r="K16" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="L16" t="n">
+      <c r="L16" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6963,10 +6963,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K17" t="n">
+      <c r="K17" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L17" s="0" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6999,10 +6999,10 @@
           <t>Partial Coverage (7/11)</t>
         </is>
       </c>
-      <c r="K18" t="n">
+      <c r="K18" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="L18" t="n">
+      <c r="L18" s="0" t="n">
         <v>4</v>
       </c>
     </row>
@@ -7039,10 +7039,10 @@
           <t>Partial Coverage (7/9)</t>
         </is>
       </c>
-      <c r="K19" t="n">
+      <c r="K19" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="L19" t="n">
+      <c r="L19" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7075,10 +7075,10 @@
           <t>Partial Coverage (5/26)</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="K20" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="L20" t="n">
+      <c r="L20" s="0" t="n">
         <v>21</v>
       </c>
     </row>
@@ -7111,10 +7111,10 @@
           <t>Partial Coverage (23/29)</t>
         </is>
       </c>
-      <c r="K21" t="n">
+      <c r="K21" s="0" t="n">
         <v>24</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L21" s="0" t="n">
         <v>5</v>
       </c>
     </row>
@@ -7151,10 +7151,10 @@
           <t>Partial Coverage (46/47)</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="K22" s="0" t="n">
         <v>46</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L22" s="0" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7184,18 +7184,14 @@
       <c r="I23" s="63" t="n"/>
       <c r="J23" s="95" t="inlineStr">
         <is>
-          <t>N/A - already covered by existing on-device script</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>TBD - Form Submissions not yet automated</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
+          <t>Partial Coverage (29/51)</t>
+        </is>
+      </c>
+      <c r="K23" s="0" t="n">
+        <v>29</v>
+      </c>
+      <c r="L23" s="0" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="24" ht="44.25" customHeight="1" s="86">
@@ -7231,10 +7227,10 @@
           <t>Partial Coverage (1/4)</t>
         </is>
       </c>
-      <c r="K24" t="n">
+      <c r="K24" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L24" s="0" t="n">
         <v>3</v>
       </c>
     </row>
@@ -7267,28 +7263,28 @@
           <t>Partial Coverage (9/24)</t>
         </is>
       </c>
-      <c r="K25" t="n">
+      <c r="K25" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L25" s="0" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="27">
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>TOTAL (excl. Form Submissions - not yet automated)</t>
-        </is>
-      </c>
-      <c r="K27" t="n">
-        <v>219</v>
-      </c>
-      <c r="L27" t="n">
-        <v>122</v>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>63.5% automated (219/345 test cases)</t>
+      <c r="B27" s="0" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="K27" s="0" t="n">
+        <v>248</v>
+      </c>
+      <c r="L27" s="0" t="n">
+        <v>143</v>
+      </c>
+      <c r="M27" s="0" t="inlineStr">
+        <is>
+          <t>63.4% automated (248/391 test cases)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Geoservices coverage, fix CI-flagged flow bugs, and sync Inventory counts
- Add flows/case_filters/geoservices_{01,02}.yaml covering the 3 previously-
  missing automatable Case Filters rows plus the automatable portion of a
  partial one, ground-truthed against the real Basic Tests CCZ.
- Fix real bugs surfaced by CI run 31476507436: commcare_odk_01_login and
  question_types_01_03 (transient dialog/timing races), setup_03 (a
  redundant back-press that exited the app), setup_05 (uninstall dialog
  button text mismatch), upload_test_01 (finish-tap race), and
  image_resize_25/26 (wrong form-structure assumption, corrected against
  the real Multimedia CCZ).
- Sync docs/Connect Test Case and Workflow Inventory.xlsx counts and
  docs/[Master] Mobile Plan (2026).xlsx notes with today's audit findings.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -6668,14 +6668,14 @@
       <c r="I9" s="45" t="n"/>
       <c r="J9" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (6/22)</t>
+          <t>Partial Coverage (21/22)</t>
         </is>
       </c>
       <c r="K9" s="0" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="L9" s="0" t="n">
-        <v>16</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="57" customHeight="1" s="86">
@@ -6780,11 +6780,11 @@
       <c r="I12" s="45" t="n"/>
       <c r="J12" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (4/13)</t>
+          <t>Partial Coverage (8/13)</t>
         </is>
       </c>
       <c r="K12" s="0" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L12" s="0" t="n">
         <v>3</v>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="J19" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (7/9)</t>
+          <t>Partial Coverage (8/9)</t>
         </is>
       </c>
       <c r="K19" s="0" t="n">
@@ -7108,11 +7108,11 @@
       <c r="I21" s="63" t="n"/>
       <c r="J21" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (23/29)</t>
+          <t>Partial Coverage (23/28)</t>
         </is>
       </c>
       <c r="K21" s="0" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="L21" s="0" t="n">
         <v>5</v>
@@ -7148,14 +7148,14 @@
       </c>
       <c r="J22" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (46/47)</t>
+          <t>Partial Coverage (44/47)</t>
         </is>
       </c>
       <c r="K22" s="0" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="L22" s="0" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" ht="39.75" customHeight="1" s="86">
@@ -7277,14 +7277,14 @@
         </is>
       </c>
       <c r="K27" s="0" t="n">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>158</v>
+        <v>145</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>59.6% automated (233/391 test cases)</t>
+          <t>63.2% automated (249/394 test cases)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document the mid-run CommCare binary-swap gap as a confirmed limitation
Investigated whether Test Cases 1/2/3/5's shared "install old APK, stage
an update, interrupt with a newer APK mid-test" precondition could be
automated. Confirmed (not just assumed, per prior sibling-flow notes in
recovery_measures) that neither Maestro nor BrowserStack App Automate/App
Live expose any API to install a new APK once a session has already
started - only an ADB-capable device farm outside BrowserStack could do
this, which is an infrastructure change, not a flow-level fix.

Documented the finding in each affected flow's header
(scenario_1/2/3/5), coverage_matrix.csv, and both tracking spreadsheets -
including correcting stale automation counts for the "Updates (partial
and failed)" tab (23/5/28 -> 24/6/30) that predated today's changes.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Connect Test Case and Workflow Inventory.xlsx
+++ b/docs/Connect Test Case and Workflow Inventory.xlsx
@@ -7108,14 +7108,14 @@
       <c r="I21" s="63" t="n"/>
       <c r="J21" s="95" t="inlineStr">
         <is>
-          <t>Partial Coverage (23/28)</t>
+          <t>Partial Coverage (24/30)</t>
         </is>
       </c>
       <c r="K21" s="0" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L21" s="0" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" ht="57" customHeight="1" s="86">
@@ -7277,14 +7277,14 @@
         </is>
       </c>
       <c r="K27" s="0" t="n">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="L27" s="0" t="n">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="M27" s="0" t="inlineStr">
         <is>
-          <t>63.2% automated (249/394 test cases)</t>
+          <t>63.1% automated (250/396 test cases)</t>
         </is>
       </c>
     </row>

</xml_diff>